<commit_message>
Leads: 2026-10-20 04:25 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>North Las Vegas HVAC Contractor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>northvegashvaccontractor.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://northvegashvaccontractor.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Service Focused</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>randy@agentboomer.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>702-343-9322</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>HVAC contractor North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 13:27 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,62 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HVAC Contractors | Kansas City, KS | McCarty Mechanical</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>mccartymechanical.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.mccartymechanical.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>mccartymechanical@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>913-432-5100</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>HVAC contractor Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 13:33 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -644,7 +644,6 @@
           <t>https://www.mccartymechanical.com/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>mccartymechanical@gmail.com</t>
@@ -674,6 +673,66 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Roofers in Boise IDAHO | Team Roofing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>teamroofingandremodelingllc.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.teamroofingandremodelingllc.com/boise-roofers</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Area Homes</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>snowfalltowingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(208) 898-9882</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>86</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roofer Boise ID</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-20 13:39 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,62 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Triple J INC.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>triplejincroofing.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://triplejincroofing.com/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>office@triplejincroofing.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>303-944-0680</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof replacement Aurora CO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 18:16 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -759,7 +759,6 @@
           <t>https://triplejincroofing.com/roof-replacement/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>office@triplejincroofing.com</t>
@@ -789,6 +788,62 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apex Roofing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>apexroofingpdx.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://apexroofingpdx.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>petrzhukivskiy@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(503) 421-1730</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roof repair company Portland OR</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-20 18:22 UTC (cycle 204)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -814,7 +814,6 @@
           <t>https://apexroofingpdx.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>petrzhukivskiy@gmail.com</t>
@@ -844,6 +843,122 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BW Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>bwairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.bwairconditioning.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>bwaced@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(954) 565-7369</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>AC installation Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Raymoore Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>yougetmoore.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://yougetmoore.com/air-conditioning-installation/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Why Indianapolis</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@yougetmoore.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(317) 418-2961</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>AC installation Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-20 18:24 UTC (cycle 205)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -869,7 +869,6 @@
           <t>https://www.bwairconditioning.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>bwaced@gmail.com</t>
@@ -959,6 +958,66 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Thomson's Roofing Company</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>thomsonroofingcompany.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.thomsonroofingcompany.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Blogs Gallery</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>john@smith.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(508) 403-1000</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Brockton MA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Brockton MA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-20</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-20 18:25 UTC (cycle 206)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Heat Wave</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>heatwavetx.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.heatwavetx.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Heat Wave</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>heatwaveac@outlook.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>469-355-4958</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Carrollton TX</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>heating and cooling company Carrollton TX</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 19:59 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1083,6 +1083,66 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Downing Plumbing</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>downingplumbing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.downingplumbing.com/service-areas/gary-in/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>County View</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>service@theduckteam.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(219) 512-9003</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumber Gary IN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 20:05 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1143,6 +1143,66 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Innovative Air</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>innovativeairhvac.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.innovativeairhvac.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Innovative Air</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>office@innovativeairhvac.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>423-557-5804</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AC installation Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 20:08 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Superior CO-OP HVAC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>scoophvac.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://scoophvac.com/heat-pumps-rutland-vt/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>What Cambridge</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@scoophvac.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(518) 333-7431</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Rutland VT</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>heat pump installation Rutland VT</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-20 20:11 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-20.xlsx
+++ b/output/leads_2026-10-20.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1263,6 +1263,122 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Wimberley Roofing</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>wimberleyroofing.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.wimberleyroofing.com/services/roofing-replacement-service</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Insurance Claim</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@wimberleyroofing.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(512) 877-0015</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roof replacement San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CDG Restoration &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>cdgaustin.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.cdgaustin.com/service-areas/san-marcos/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@cdgaustin.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(737) 309-5075</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roof replacement San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>